<commit_message>
WIP bumping XLSXasJSON and JSON
</commit_message>
<xml_diff>
--- a/test/project/xlsx/Folder/Character.xlsx
+++ b/test/project/xlsx/Folder/Character.xlsx
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr fullCalcOnLoad="1" calcMode="auto"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Key</t>
   </si>
@@ -70,6 +70,24 @@
   </si>
   <si>
     <t>$UIText/2</t>
+  </si>
+  <si>
+    <t>/Key</t>
+  </si>
+  <si>
+    <t>/$UIText</t>
+  </si>
+  <si>
+    <t>Bard sings ;a song, but doesn't dance</t>
+  </si>
+  <si>
+    <t>Wizard can cast;a spell</t>
+  </si>
+  <si>
+    <t>Warrior yields;the sword</t>
+  </si>
+  <si>
+    <t>Archer fire arrows;with a bow</t>
   </si>
 </sst>
 </file>
@@ -401,27 +419,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:D5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="17.42578125" customWidth="1"/>
     <col min="4" max="4" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s" s="1">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
         <v>10</v>
@@ -430,9 +454,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -441,9 +468,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
@@ -452,9 +482,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Enhance json_to_xl functionality: add support for preserving existing Excel headers and indexed-array expansion in json_to_xl_headers
</commit_message>
<xml_diff>
--- a/test/project/xlsx/Folder/Character.xlsx
+++ b/test/project/xlsx/Folder/Character.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="22">
   <si>
     <t>Key</t>
   </si>
@@ -88,6 +88,9 @@
   </si>
   <si>
     <t>Archer fire arrows;with a bow</t>
+  </si>
+  <si>
+    <t>/$UIText/3</t>
   </si>
 </sst>
 </file>
@@ -431,13 +434,13 @@
         <v>15</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s" s="1">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>